<commit_message>
Updated actual cost of oredered parts.
</commit_message>
<xml_diff>
--- a/Cost.xlsx
+++ b/Cost.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\matthias\Documents\bike-light-rear\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C3C732-819D-4EAB-8826-880399D132F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49FEA58E-AF7B-46FA-941B-CF1DE93138AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Column1</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Cost [€]</t>
   </si>
   <si>
-    <t>Parts Excluded from BOM</t>
-  </si>
-  <si>
     <t>USB4105-GF-A-060</t>
   </si>
   <si>
@@ -99,6 +96,18 @@
   </si>
   <si>
     <t>OPT3001DNPR</t>
+  </si>
+  <si>
+    <t>Parts Excluded from BOM (excl. TAX)</t>
+  </si>
+  <si>
+    <t>Tariffs (JLCPCB)</t>
+  </si>
+  <si>
+    <t>TAX (Digikey)</t>
+  </si>
+  <si>
+    <t>Price for Only 5 pcs</t>
   </si>
 </sst>
 </file>
@@ -441,8 +450,9 @@
   <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="22.9296875" customWidth="1"/>
-    <col min="2" max="4" width="10.1328125" customWidth="1"/>
+    <col min="1" max="1" width="31.86328125" customWidth="1"/>
+    <col min="2" max="3" width="10.1328125" customWidth="1"/>
+    <col min="4" max="4" width="17.06640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -461,7 +471,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
@@ -469,25 +479,25 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>0.5</v>
+        <v>0.434</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4">
-        <v>3.9550000000000001</v>
+        <v>2.6619999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0.56899999999999995</v>
@@ -495,7 +505,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>0.21</v>
@@ -503,15 +513,18 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9">
-        <v>8.07</v>
+        <v>3.71</v>
+      </c>
+      <c r="D9" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10">
         <v>5.27</v>
@@ -519,7 +532,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11">
         <v>0.29699999999999999</v>
@@ -527,7 +540,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>1.4930000000000001</v>
@@ -535,7 +548,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13">
         <v>1.0860000000000001</v>
@@ -543,7 +556,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14">
         <v>1.6759999999999999</v>
@@ -551,15 +564,32 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17">
-        <v>9</v>
+        <v>8.68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18">
+        <v>7.93</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19">
+        <f>SUM(B7:B15)*B24*0.2</f>
+        <v>28.622000000000003</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
@@ -568,7 +598,7 @@
       </c>
       <c r="B23">
         <f>SUM(B3:B15)+SUM(B17:B21)/B24</f>
-        <v>24.025999999999993</v>
+        <v>21.930199999999999</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
@@ -585,7 +615,7 @@
       </c>
       <c r="B25">
         <f>B23*B24</f>
-        <v>240.25999999999993</v>
+        <v>219.30199999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>